<commit_message>
MLB 2026-04-04 Run 2: full pipeline — Griffin debut, Braves 17-2, Kirk injury, Ohtani April 8
7 stories, 8 X posts, 5 articles, PostPlanner exports, review dashboard published.
Key stories: Konnor Griffin MLB debut RBI double (youngest SS since A-Rod 1994), Braves 17-2 AZ,
Alejandro Kirk thumb fracture 6-8 weeks, Giants 7-2 Mets, Ohtani April 8 pitching start,
early season standings (Yankees/Marlins/Brewers 5-1), Sunday preview.

https://claude.ai/code/session_0178Pb7ZnrqGqbWCLboPEiPL
</commit_message>
<xml_diff>
--- a/MLB/postplanner-imports/bb-postplanner-2026-04-04.xlsx
+++ b/MLB/postplanner-imports/bb-postplanner-2026-04-04.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,333 +478,121 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>04/04/2026  17:26</t>
+          <t>04/04/2026  18:52</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Aaron Judge homered in the FIRST AT-BAT of the Yankees' home opener Friday.
-HR No. 371. Passes Hall of Famer Gil Hodges (83rd all-time).
-2-run shot. 387 feet. 101 mph. Off Eury Perez.
-Yankees win 8-2. New York is 6-1. Best record in the AL.
-#Yankees #MLB</t>
+          <t>Konnor Griffin. First MLB at-bat. RBI double. 105.8 mph. 369 feet.
+He is 19 years old. He is the youngest shortstop to debut in MLB since Alex Rodriguez in 1994.
+The hype was real. #LetsGoBucs #Pirates #MLB</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>04/04/2026  17:41</t>
+          <t>04/04/2026  19:15</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Aaron Judge wanted to make a statement at Yankee Stadium's home opener — and he delivered before most fans had finished their first hot dog.
-On his very first at-bat of the home opener on Friday, Judge drove a slider from Marlins right-hander Eury Perez 387 feet to left field, 101.2 mph off the bat, for a 2-run home run. It was career home run No. 371 for the Yankees captain, moving him past Hall of Famer Gil Hodges into sole possession of 83rd place on the all-time home run list.
-Three home runs in seven games to open 2026. The Yankees beat the Marlins 8-2 to improve to 6-1 on the season — the best record in the American League. New York looks like a team that isn't just competitive but dominant, and Judge is producing exactly as advertised.
-At 371 career home runs at age 34, Judge's path to 400 — a milestone that would cement his place among the all-time greats — is a genuine storyline to track all season. He needs 29 more to reach that mark.</t>
+          <t>Sunday in baseball:
+• Braves go for the sweep over AZ
+• Pirates look for back-to-back behind Griffin
+• Series finales across the league
+And then Tuesday: Shohei Ohtani on the mound again.
+One of the best weeks in baseball ahead. ⚾ #MLB</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>04/04/2026  17:56</t>
+          <t>04/04/2026  19:38</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>HR No. 371. First at-bat of the home opener. Aaron Judge passed Hall of Famer Gil Hodges (83rd all-time) on Friday. Yankees 8-2. New York is 6-1. #Yankees #MLB</t>
+          <t>Pirates home opener recap:
+🏠 PNC Park sold out (~38,986 fans)
+✅ Konnor Griffin: RBI double in 1st AB, 2 runs scored
+✅ Pirates win 5-4 over Baltimore
+The No. 1 prospect did not disappoint. #LetsGoBucs #KonnorGriffin</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04/04/2026  18:11</t>
+          <t>04/04/2026  20:01</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yankees 6-1. Best record in the American League.
-Aaron Judge: 3 HRs in 7 games. 371 career. 29 from 400.
-This team is already rolling. #Yankees</t>
+          <t>The Braves are awake.
+Atlanta 17, Arizona 2.
+17 runs. Saturdays are for statement games. #Braves #Atlanta #MLB</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04/04/2026  18:26</t>
+          <t>04/04/2026  20:24</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Shohei Ohtani hit his first HR of 2026 Friday.
-3-run shot in the 3rd inning. Dodgers score 10 straight. Win 13-6.
-Kyle Tucker also homered — first as a Dodger.
-5 total LA HRs. Ohtani's on-base streak is now at 38 straight games.
-#Dodgers #MLB</t>
+          <t>Mark your calendars: Shohei Ohtani pitches again TUESDAY, April 8, vs. the Blue Jays.
+He went 6 scoreless innings in his 2026 debut (March 31). Then hit his first HR of the year April 3.
+The two-way season is absolutely happening. #Dodgers #Ohtani #MLB</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04/04/2026  18:41</t>
+          <t>04/04/2026  20:47</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>It took seven games, but Shohei Ohtani is officially in the home run column for 2026.
-Ohtani launched a 3-run shot in the third inning of the Dodgers' 13-6 demolition of Washington on Friday, sparking a 10-run response from a lineup that looks genuinely dangerous. Kyle Tucker added his first home run as a Dodger, Mookie Betts homered, and Freddie Freeman hit a 2-run shot — five total Los Angeles home runs in the rout.
-Starter Emmett Sheehan earned the win with 5.2 innings of work. On the other side, Miles Mikolas had an ugly afternoon, allowing a career-high 11 runs in just 4.1 innings.
-The eye-catching number? Ohtani's on-base streak now sits at 38 consecutive games, dating back to last season. His 2026 season as a two-way player is just getting started, and this is what it looks like when everything clicks offensively.
-The Dodgers are 4-2 after seven games — exactly the kind of start their World Series hopes require.</t>
+          <t>Not good news for the Blue Jays.
+Alejandro Kirk fractured and dislocated his thumb on a foul tip. Could miss 6-8 weeks if surgery is required.
+Brandon Valenzuela recalled. Toronto hoping for the best. #BlueJays #MLB</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04/04/2026  18:56</t>
+          <t>04/04/2026  21:10</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ohtani's first HR of 2026. Tucker's first as a Dodger. Five total LA HRs. Dodgers 13, Nationals 6. Ohtani's on-base streak: 38 straight games. #Dodgers #MLB</t>
+          <t>Giants 7, Mets 2.
+San Francisco winning on Saturday. New York can't buy consistency right now.
+The NL East race is anything but settled. #SFGiants #Mets #MLB</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04/04/2026  19:11</t>
+          <t>04/04/2026  21:33</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Chase DeLauter has 5 HRs in 7 career MLB games.
-He's only the 4th player in history to do it — Trevor Story, Mark Quinn, Rece Hinds.
-Friday: 2-run blast, 402 feet. Guardians beat the Cubs 4-1 in the home opener.
-This kid is different. #ClevelandGuardians #MLB</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>04/04/2026  19:26</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Minnesota home opener.
-Twins trailed the Rays heading into the 7th, then erupted for SEVEN runs.
-Tristan Gray grand slam. Final: Twins 10, Rays 4.
-Tampa Bay falls to 2-4. Not the start they wanted. #Twins #Rays #MLB</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>04/04/2026  19:41</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Chase DeLauter's start to his MLB career is not normal.
-On Friday night, the Cleveland Guardians outfielder ripped his 5th home run in only his 7th career regular-season game — a 2-run blast off Hunter Harvey that traveled 402 feet, helping Cleveland beat the Cubs 4-1 in their home opener. DeLauter went 3-for-4.
-Here's the historical context: only three other players in MLB history have hit 5 or more home runs in their first seven career regular-season games. The list is Trevor Story (Colorado, 2016), Mark Quinn (Kansas City, 1999), and Rece Hinds (Cincinnati, 2024). DeLauter is now in that company.
-He is tied for the American League home run lead with five big flies in seven games. This is not a hot streak — this looks like something else entirely.
-The Guardians are 4-3 on the season, and their most electric story is just getting started.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>04/04/2026  19:56</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Chase DeLauter has 5 HRs in 7 career MLB games — only the 4th player in history to do it. Guardians beat the Cubs 4-1 in Friday's home opener. #ClevelandGuardians #MLB</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>04/04/2026  20:11</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Minnesota fans at Target Field got exactly what they came for in the home opener on Friday.
-The Twins trailed entering the seventh inning, then exploded for seven runs in the frame — capped by a Tristan Gray grand slam — to pull away from Tampa Bay and win 10-4. It was the kind of comeback inning that gets a home crowd on its feet and sets the tone for a season.
-The Rays fell to 2-4 with the loss. Tampa Bay has been one of baseball's most reliable franchises over the past decade, but this early-April slide will need to stop before the American League standings start looking ominous.
-The Twins, meanwhile, have something to build on as they look to claw their way back to relevance in the AL Central.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>04/04/2026  20:26</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Tristan Gray grand slam highlights a 7-run 7th inning as the Twins top the Rays 10-4 in Friday's home opener. Tampa falls to 2-4. #Twins #Rays #MLB</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>04/04/2026  20:41</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Guardians 4-1 over the Cubs in their home opener Friday.
-Chase DeLauter: 3-for-4. HR No. 5. 402 feet.
-Tied for the AL HR lead in just 7 career games.
-Cleveland is building something real. #ClevelandGuardians</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>04/04/2026  20:56</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>The 2026 rookie class Week 1:
-DeLauter + Stewart won both first POTWs (only 2nd time ever both went to rookies).
-Murakami HR in first 3 games. McGonigle 4-hit debut. Wetherholt walk-off.
-The future is now. #MLB</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>04/04/2026  21:11</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>It is fair to say that no rookie class has opened a season quite like the 2026 group.
-Here's the Week 1 résumé: Chase DeLauter hit 5 home runs in his first 7 career games — only the 4th player in MLB history to do so. Munetaka Murakami (Chicago White Sox) homered in each of his first three MLB games, making him only the third or fourth player ever to accomplish that. Aaron Stewart (Cincinnati Reds) hit .700 in his first week and won the NL Player of the Week award. DeLauter claimed the AL honor.
-That's only the second time in MLB history that both first weekly awards of the season went to rookies. The last time? 2016, when Trevor Story and Tyler White pulled it off.
-Meanwhile, Kevin McGonigle (Detroit Tigers) had four hits in his MLB debut — the third-youngest player in the past 100 years to accomplish that. Jackson Wetherholt (St. Louis Cardinals) delivered a walk-off home run. Carson Benge (New York Mets) hit a home run and stole a base in his debut.
-Six rookies. Six remarkable stories. All in the first seven days of the season. This class is one to watch all year.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>04/04/2026  21:26</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>DeLauter + Stewart both won Week 1 POTWs — only the 2nd time in MLB history both first awards went to rookies. Murakami HR in first 3 games. What a rookie class. #MLB #Baseball</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>04/04/2026  21:41</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Early 2026 MLB standings:
-AL: Yankees 6-1 | Astros 5-2 | Blue Jays 4-2
-NL: Brewers 5-1 | Marlins 5-2 | Braves 5-2
-White Sox and Red Sox both at 1-5.
-A's 1-5 too.
-Seven games in. It's still early. But some patterns are forming. #MLB</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>04/04/2026  21:56</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Seven games into the 2026 MLB season, some teams are already separating themselves. Here's where things stand:
-American League:
-The Yankees lead the AL at 6-1 — the best record in the league. Houston (5-2) is right behind them. The Blue Jays (4-2) are quietly in the hunt. At the bottom: the White Sox and Red Sox are both at 1-5 after a week. The Athletics are 1-5 as well.
-National League:
-Milwaukee leads the NL Central at 5-1. Miami (5-2) and Atlanta (5-2) are locked in an early NL East race. The Dodgers sit at 4-2 in the NL West, having recovered from a rough series against Cleveland.
-Teams to watch: The Guardians are 4-3 but own the most electrifying hitter in the sport right now in DeLauter. Pittsburgh (3-3) is still adjusting to life with their top prospect Griffin in the lineup.
-It's still early — way too early to draw conclusions. But the early-season trends are worth noting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>04/04/2026  22:11</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Early 2026 MLB standings: Yankees 6-1 lead AL. Brewers 5-1 lead NL Central. Marlins + Braves 5-2 in NL East. White Sox + Red Sox + A's all at 1-5. #MLB #Baseball</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>04/04/2026  22:26</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Full Saturday MLB slate today.
-Yankees-Marlins G3. Dodgers-Nationals G3. Guardians-Cubs G3.
-Twins-Rays wrapping up. Red Sox-Padres series continues.
-38 teams. 15 games. One league. #MLB #Baseball</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>04/04/2026  22:41</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>After Friday's fireworks — Judge's first-AB homer, DeLauter's 5th, Ohtani's first bomb of 2026, and a Twins home opener explosion — Saturday gives us a full schedule of action to follow.
-Key matchups to watch: The Yankees and Marlins wrap up their series in New York. The Dodgers and Nationals close out in Washington. The Guardians and Cubs finish their home stand in Cleveland. Plus Red Sox-Padres, Cardinals-Tigers, Reds-Rangers, and several other series finales.
-After seven games, the landscape is taking shape. Starting pitching matchups get better every week, rosters settle in, and the patterns of a 162-game season begin to emerge.
-Baseball is back and it is very, very good.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>04/04/2026  22:56</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Full Saturday slate: Yankees-Marlins G3. Dodgers-Nationals G3. Guardians-Cubs G3. Plus a dozen more. Week 1 wrapping up — what a start to 2026. #MLB #Baseball</t>
+          <t>Early-season MLB standings check:
+🗽 Yankees: 5-1 (AL East)
+🐟 Marlins: 5-1 (NL East)
+🍺 Brewers: 5-1 (NL Central)
+⚾ Dodgers: 4-2 (NL West)
+🚀 Astros: 5-2 (AL West)
+Miami leading the NL East. The chaos has begun. #MLB #BaseballIsBack</t>
         </is>
       </c>
     </row>

</xml_diff>